<commit_message>
Field outline workbook: payer classes 1-7, top 5 payers, planned changes per source
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rd4bPes2nDH7UjsCQMWVQG
</commit_message>
<xml_diff>
--- a/docs/provider-directory-field-outline.xlsx
+++ b/docs/provider-directory-field-outline.xlsx
@@ -887,7 +887,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Approximate age, estimated from medical school graduation year. Not a date of birth.</t>
+          <t>Approximate age, estimated from medical school graduation year.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>1 when any cms_pdc_facility_affil row exists for the NPI (PDC Facility Affiliation dataset 27ea-46a8). pd_network_npi holds the CCNs. Not a contracted-network flag.</t>
+          <t>1 when any cms_pdc_facility_affil row exists for the NPI (PDC Facility Affiliation dataset 27ea-46a8). pd_network_npi holds the CCNs.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>* Total-RVU scale, one work procedure per visit. Not a CMS physician work RVU report.
+          <t>* Fee-schedule RVU, one procedure per visit, under review.
 * Visits whose procedure has no fee-schedule RVU are excluded.</t>
         </is>
       </c>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>* Total-RVU scale, one work procedure per visit. Not a CMS physician work RVU report.
+          <t>* Fee-schedule RVU, one procedure per visit, under review.
 * Peers are same-specialty clinicians with a positive RVU total.</t>
         </is>
       </c>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Total-RVU scale, one work procedure per visit. Not a CMS physician work RVU report.</t>
+          <t>Fee-schedule RVU, one procedure per visit, under review.</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Total-RVU scale, one work procedure per visit. Not a CMS physician work RVU report.</t>
+          <t>Fee-schedule RVU, one procedure per visit, under review.</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>* Total-RVU scale, one work procedure per visit. Not a CMS physician work RVU report.
+          <t>* Fee-schedule RVU, one procedure per visit, under review.
 * Visits whose procedure has no fee-schedule RVU are excluded.</t>
         </is>
       </c>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals. Not stored; shares of all visits, so the three do not add to 100.</t>
+          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals, computed at read time. Shares of all visits, so the three do not add to 100.</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals. Not stored; shares of all visits, so the three do not add to 100.</t>
+          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals, computed at read time. Shares of all visits, so the three do not add to 100.</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals. Not stored; shares of all visits, so the three do not add to 100.</t>
+          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals, computed at read time. Shares of all visits, so the three do not add to 100.</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals. Not stored; shares of all visits, so the three do not add to 100.</t>
+          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals, computed at read time. Shares of all visits, so the three do not add to 100.</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals. Not stored; shares of all visits, so the three do not add to 100.</t>
+          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals, computed at read time. Shares of all visits, so the three do not add to 100.</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
@@ -3144,7 +3144,7 @@
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals. Not stored; shares of all visits, so the three do not add to 100.</t>
+          <t>Computed at read time: pd_stg_top_dx / pd_stg_top_px visit_count / pd_provider.visits_total x100, 2 decimals, computed at read time. Shares of all visits, so the three do not add to 100.</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>* Total-RVU scale, one work procedure per visit. Not a CMS physician work RVU report.
+          <t>* Fee-schedule RVU, one procedure per visit, under review.
 * Visits whose procedure has no fee-schedule RVU are excluded.</t>
         </is>
       </c>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Total-RVU scale, one work procedure per visit. Not a CMS physician work RVU report.</t>
+          <t>Fee-schedule RVU, one procedure per visit, under review.</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">

</xml_diff>